<commit_message>
pruebas: Gerencia - Excel mensuales actualizados a Septiembre 2026
Publica en /pruebas/ los datos de develop (76c6933) del repo privado:
COMPRAS.xlsx, DETALLE POR PROVEEDOR.xlsx, INVENTARIO POR MESES.xlsx,
INVENTARIO.xlsx, TABLERO.xlsx, TALENTO HUMANO.xlsx, VENTAS.csv y datos.xlsx.
Sin cambios de codigo. /oficial/ no se toca.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pruebas/Gerencia/DETALLE POR PROVEEDOR.xlsx
+++ b/pruebas/Gerencia/DETALLE POR PROVEEDOR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ade4bf4107253254/OPAUSTRO DASHBOARD/TI OPAUSTRO/APP OPAUSTRO/APP OPAUSTRO/Gerencia/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ade4bf4107253254/OPAUSTRO DASHBOARD/TI OPAUSTRO/CLAUDE/APP OPAUSTRO/Gerencia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="727" documentId="8_{0430E75C-45C4-434B-A5FC-9A7906183C89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1435C302-0E05-4C9C-9998-5A9C19862744}"/>
+  <xr:revisionPtr revIDLastSave="811" documentId="8_{0430E75C-45C4-434B-A5FC-9A7906183C89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7630B9F4-58E8-4144-B9B3-54A84C574B3D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{648B2FA4-D191-4427-B2D8-D6C121F05EA1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{648B2FA4-D191-4427-B2D8-D6C121F05EA1}"/>
   </bookViews>
   <sheets>
     <sheet name="POR LINEA" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="874" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="982" uniqueCount="26">
   <si>
     <t>Suma de VentaNeta</t>
   </si>
@@ -118,6 +118,9 @@
   </si>
   <si>
     <t>VALOR</t>
+  </si>
+  <si>
+    <t>SEPTIEMBRE</t>
   </si>
 </sst>
 </file>
@@ -518,22 +521,44 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="8">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{D96A059A-F05F-4659-BFA4-F4A26AEA1E86}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;8262c8bf-4a44-4c82-8dcf-5713f882f648&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A73EA3A-E1FE-485B-B71A-B3ECBB4FF369}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:I241"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I272"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="28.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.109375" customWidth="1"/>
-    <col min="6" max="6" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.44140625" customWidth="1"/>
-    <col min="8" max="8" width="61.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.140625" customWidth="1"/>
+    <col min="6" max="6" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" customWidth="1"/>
+    <col min="8" max="8" width="61.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -550,7 +575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2026</v>
       </c>
@@ -567,7 +592,7 @@
         <v>85495.516999998275</v>
       </c>
     </row>
-    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2026</v>
       </c>
@@ -584,7 +609,7 @@
         <v>92851.959499999793</v>
       </c>
     </row>
-    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -601,7 +626,7 @@
         <v>133348.79079999981</v>
       </c>
     </row>
-    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2026</v>
       </c>
@@ -618,7 +643,7 @@
         <v>249594.42229999453</v>
       </c>
     </row>
-    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2026</v>
       </c>
@@ -635,7 +660,7 @@
         <v>721989.16590005404</v>
       </c>
     </row>
-    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2026</v>
       </c>
@@ -652,7 +677,7 @@
         <v>189198.49</v>
       </c>
     </row>
-    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2026</v>
       </c>
@@ -670,7 +695,7 @@
         <v>82262.724100000705</v>
       </c>
     </row>
-    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2026</v>
       </c>
@@ -688,7 +713,7 @@
         <v>78760.872100000503</v>
       </c>
     </row>
-    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2026</v>
       </c>
@@ -706,7 +731,7 @@
         <v>93186.947200008013</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2026</v>
       </c>
@@ -724,7 +749,7 @@
         <v>204233.279800007</v>
       </c>
     </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2026</v>
       </c>
@@ -742,7 +767,7 @@
         <v>508684.41419994994</v>
       </c>
     </row>
-    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2026</v>
       </c>
@@ -759,7 +784,7 @@
         <v>156678.5</v>
       </c>
     </row>
-    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2026</v>
       </c>
@@ -776,7 +801,7 @@
         <v>10670.3213</v>
       </c>
     </row>
-    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2026</v>
       </c>
@@ -793,7 +818,7 @@
         <v>11697.601199999999</v>
       </c>
     </row>
-    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2026</v>
       </c>
@@ -810,7 +835,7 @@
         <v>23058.0075</v>
       </c>
     </row>
-    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2026</v>
       </c>
@@ -827,7 +852,7 @@
         <v>29808.748900000002</v>
       </c>
     </row>
-    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2026</v>
       </c>
@@ -844,7 +869,7 @@
         <v>119133.63</v>
       </c>
     </row>
-    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2026</v>
       </c>
@@ -861,7 +886,7 @@
         <v>37362.78</v>
       </c>
     </row>
-    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2026</v>
       </c>
@@ -878,7 +903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2026</v>
       </c>
@@ -895,7 +920,7 @@
         <v>711.53110000000004</v>
       </c>
     </row>
-    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2026</v>
       </c>
@@ -912,7 +937,7 @@
         <v>2363.2370000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2026</v>
       </c>
@@ -929,7 +954,7 @@
         <v>4434.2187999999996</v>
       </c>
     </row>
-    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2026</v>
       </c>
@@ -946,7 +971,7 @@
         <v>32310.115500000007</v>
       </c>
     </row>
-    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2026</v>
       </c>
@@ -963,7 +988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2026</v>
       </c>
@@ -980,7 +1005,7 @@
         <v>77493.450099998765</v>
       </c>
     </row>
-    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2026</v>
       </c>
@@ -997,7 +1022,7 @@
         <v>76674.18439999946</v>
       </c>
     </row>
-    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2026</v>
       </c>
@@ -1014,7 +1039,7 @@
         <v>145359.8761000009</v>
       </c>
     </row>
-    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>2026</v>
       </c>
@@ -1031,7 +1056,7 @@
         <v>270902.51149999269</v>
       </c>
     </row>
-    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2026</v>
       </c>
@@ -1048,7 +1073,7 @@
         <v>662560.93030006299</v>
       </c>
     </row>
-    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2026</v>
       </c>
@@ -1065,7 +1090,7 @@
         <v>182425.68</v>
       </c>
     </row>
-    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2026</v>
       </c>
@@ -1083,7 +1108,7 @@
         <v>65610.900000000009</v>
       </c>
     </row>
-    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2026</v>
       </c>
@@ -1101,7 +1126,7 @@
         <v>64001.93</v>
       </c>
     </row>
-    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2026</v>
       </c>
@@ -1119,7 +1144,7 @@
         <v>136910.14000000001</v>
       </c>
     </row>
-    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2026</v>
       </c>
@@ -1137,7 +1162,7 @@
         <v>229309.49</v>
       </c>
     </row>
-    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>2026</v>
       </c>
@@ -1155,7 +1180,7 @@
         <v>518337.7</v>
       </c>
     </row>
-    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>2026</v>
       </c>
@@ -1173,7 +1198,7 @@
         <v>151210.75</v>
       </c>
     </row>
-    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>2026</v>
       </c>
@@ -1190,7 +1215,7 @@
         <v>10531.8115</v>
       </c>
     </row>
-    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2026</v>
       </c>
@@ -1207,7 +1232,7 @@
         <v>11559.706</v>
       </c>
     </row>
-    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>2026</v>
       </c>
@@ -1224,7 +1249,7 @@
         <v>22468.162499999999</v>
       </c>
     </row>
-    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>2026</v>
       </c>
@@ -1241,7 +1266,7 @@
         <v>29646.756300000001</v>
       </c>
     </row>
-    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>2026</v>
       </c>
@@ -1258,7 +1283,7 @@
         <v>115484.54</v>
       </c>
     </row>
-    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>2026</v>
       </c>
@@ -1275,7 +1300,7 @@
         <v>39868.39</v>
       </c>
     </row>
-    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>2026</v>
       </c>
@@ -1292,7 +1317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>2026</v>
       </c>
@@ -1309,7 +1334,7 @@
         <v>584.46839999999997</v>
       </c>
     </row>
-    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>2026</v>
       </c>
@@ -1326,7 +1351,7 @@
         <v>3877.0530000000003</v>
       </c>
     </row>
-    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>2026</v>
       </c>
@@ -1343,7 +1368,7 @@
         <v>7465.2200999999995</v>
       </c>
     </row>
-    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2026</v>
       </c>
@@ -1360,7 +1385,7 @@
         <v>19470.09</v>
       </c>
     </row>
-    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>2026</v>
       </c>
@@ -1377,7 +1402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>2026</v>
       </c>
@@ -1394,7 +1419,7 @@
         <v>94603.869499997993</v>
       </c>
     </row>
-    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>2026</v>
       </c>
@@ -1411,7 +1436,7 @@
         <v>95555.474599999463</v>
       </c>
     </row>
-    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>2026</v>
       </c>
@@ -1428,7 +1453,7 @@
         <v>144129.24850000211</v>
       </c>
     </row>
-    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>2026</v>
       </c>
@@ -1445,7 +1470,7 @@
         <v>269266.57749999734</v>
       </c>
     </row>
-    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>2026</v>
       </c>
@@ -1463,7 +1488,7 @@
         <v>743534.1</v>
       </c>
     </row>
-    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>2026</v>
       </c>
@@ -1480,7 +1505,7 @@
         <v>231148.11</v>
       </c>
     </row>
-    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>2026</v>
       </c>
@@ -1498,7 +1523,7 @@
         <v>86602.360000001296</v>
       </c>
     </row>
-    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>2026</v>
       </c>
@@ -1516,7 +1541,7 @@
         <v>78905.321900002105</v>
       </c>
     </row>
-    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>2026</v>
       </c>
@@ -1534,7 +1559,7 @@
         <v>127594.21980000602</v>
       </c>
     </row>
-    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>2026</v>
       </c>
@@ -1552,7 +1577,7 @@
         <v>216005.05070000701</v>
       </c>
     </row>
-    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>2026</v>
       </c>
@@ -1570,7 +1595,7 @@
         <v>596867.74390001304</v>
       </c>
     </row>
-    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>2026</v>
       </c>
@@ -1587,7 +1612,7 @@
         <v>192704.66</v>
       </c>
     </row>
-    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>2026</v>
       </c>
@@ -1604,7 +1629,7 @@
         <v>10557.191500000001</v>
       </c>
     </row>
-    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>2026</v>
       </c>
@@ -1621,7 +1646,7 @@
         <v>11532.108</v>
       </c>
     </row>
-    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>2026</v>
       </c>
@@ -1638,7 +1663,7 @@
         <v>23677.612500000003</v>
       </c>
     </row>
-    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>2026</v>
       </c>
@@ -1655,7 +1680,7 @@
         <v>28823.721600000004</v>
       </c>
     </row>
-    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>2026</v>
       </c>
@@ -1672,7 +1697,7 @@
         <v>111472.32000000001</v>
       </c>
     </row>
-    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>2026</v>
       </c>
@@ -1689,7 +1714,7 @@
         <v>41922.99</v>
       </c>
     </row>
-    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>2026</v>
       </c>
@@ -1706,7 +1731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>2026</v>
       </c>
@@ -1723,7 +1748,7 @@
         <v>736.35030000000006</v>
       </c>
     </row>
-    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>2026</v>
       </c>
@@ -1740,7 +1765,7 @@
         <v>5370.5995000000012</v>
       </c>
     </row>
-    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>2026</v>
       </c>
@@ -1757,7 +1782,7 @@
         <v>6051.3029999999999</v>
       </c>
     </row>
-    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>2026</v>
       </c>
@@ -1774,7 +1799,7 @@
         <v>17917.3999</v>
       </c>
     </row>
-    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>2026</v>
       </c>
@@ -1791,7 +1816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>2026</v>
       </c>
@@ -1808,7 +1833,7 @@
         <v>80338.175099998902</v>
       </c>
     </row>
-    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>2026</v>
       </c>
@@ -1825,7 +1850,7 @@
         <v>99054.254999999743</v>
       </c>
     </row>
-    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>2026</v>
       </c>
@@ -1842,7 +1867,7 @@
         <v>140509.35320000048</v>
       </c>
     </row>
-    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>2026</v>
       </c>
@@ -1859,7 +1884,7 @@
         <v>278723.60909999692</v>
       </c>
     </row>
-    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>2026</v>
       </c>
@@ -1876,7 +1901,7 @@
         <v>760354.35000000009</v>
       </c>
     </row>
-    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>2026</v>
       </c>
@@ -1893,7 +1918,7 @@
         <v>233588.95</v>
       </c>
     </row>
-    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>2026</v>
       </c>
@@ -1911,7 +1936,7 @@
         <v>76133.7794999998</v>
       </c>
     </row>
-    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>2026</v>
       </c>
@@ -1929,7 +1954,7 @@
         <v>84075.149199999592</v>
       </c>
     </row>
-    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>2026</v>
       </c>
@@ -1947,7 +1972,7 @@
         <v>117670.97500000801</v>
       </c>
     </row>
-    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>2026</v>
       </c>
@@ -1965,7 +1990,7 @@
         <v>262451.75289999903</v>
       </c>
     </row>
-    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>2026</v>
       </c>
@@ -1983,7 +2008,7 @@
         <v>581180.05000000005</v>
       </c>
     </row>
-    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>2026</v>
       </c>
@@ -2000,7 +2025,7 @@
         <v>179466.4</v>
       </c>
     </row>
-    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>2026</v>
       </c>
@@ -2017,7 +2042,7 @@
         <v>11075.442200000001</v>
       </c>
     </row>
-    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>2026</v>
       </c>
@@ -2034,7 +2059,7 @@
         <v>12081.7032</v>
       </c>
     </row>
-    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>2026</v>
       </c>
@@ -2051,7 +2076,7 @@
         <v>25183.904999999999</v>
       </c>
     </row>
-    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>2026</v>
       </c>
@@ -2068,7 +2093,7 @@
         <v>29972.369600000002</v>
       </c>
     </row>
-    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>2026</v>
       </c>
@@ -2085,7 +2110,7 @@
         <v>122623.67000000001</v>
       </c>
     </row>
-    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>2026</v>
       </c>
@@ -2102,7 +2127,7 @@
         <v>46622.87</v>
       </c>
     </row>
-    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>2026</v>
       </c>
@@ -2119,7 +2144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>2026</v>
       </c>
@@ -2136,7 +2161,7 @@
         <v>510.22829999999999</v>
       </c>
     </row>
-    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>2026</v>
       </c>
@@ -2153,7 +2178,7 @@
         <v>4158.4265999999998</v>
       </c>
     </row>
-    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>2026</v>
       </c>
@@ -2170,7 +2195,7 @@
         <v>3154.4038999999998</v>
       </c>
     </row>
-    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>2026</v>
       </c>
@@ -2188,7 +2213,7 @@
         <v>24851.304100000001</v>
       </c>
     </row>
-    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>2026</v>
       </c>
@@ -2205,7 +2230,7 @@
         <v>46.087000000000003</v>
       </c>
     </row>
-    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>2026</v>
       </c>
@@ -2222,7 +2247,7 @@
         <v>76043.719299999633</v>
       </c>
     </row>
-    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>2026</v>
       </c>
@@ -2239,7 +2264,7 @@
         <v>94806.232200000159</v>
       </c>
     </row>
-    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>2026</v>
       </c>
@@ -2256,7 +2281,7 @@
         <v>154992.7959999984</v>
       </c>
     </row>
-    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>2026</v>
       </c>
@@ -2273,7 +2298,7 @@
         <v>282588.31710000057</v>
       </c>
     </row>
-    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>2026</v>
       </c>
@@ -2290,7 +2315,7 @@
         <v>755337.35</v>
       </c>
     </row>
-    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>2026</v>
       </c>
@@ -2307,7 +2332,7 @@
         <v>232957.97</v>
       </c>
     </row>
-    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>2026</v>
       </c>
@@ -2325,7 +2350,7 @@
         <v>71335.639599999398</v>
       </c>
     </row>
-    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>2026</v>
       </c>
@@ -2343,7 +2368,7 @@
         <v>78424.835600000108</v>
       </c>
     </row>
-    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>2026</v>
       </c>
@@ -2361,7 +2386,7 @@
         <v>104650.97910000899</v>
       </c>
     </row>
-    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>2026</v>
       </c>
@@ -2379,7 +2404,7 @@
         <v>189148.86240000301</v>
       </c>
     </row>
-    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>2026</v>
       </c>
@@ -2397,7 +2422,7 @@
         <v>537816.41999999993</v>
       </c>
     </row>
-    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>2026</v>
       </c>
@@ -2414,7 +2439,7 @@
         <v>185918.23</v>
       </c>
     </row>
-    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>2026</v>
       </c>
@@ -2431,7 +2456,7 @@
         <v>13345.494999999999</v>
       </c>
     </row>
-    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>2026</v>
       </c>
@@ -2448,7 +2473,7 @@
         <v>14643.776</v>
       </c>
     </row>
-    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>2026</v>
       </c>
@@ -2465,7 +2490,7 @@
         <v>28558.537500000002</v>
       </c>
     </row>
-    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>2026</v>
       </c>
@@ -2482,7 +2507,7 @@
         <v>37499.223299999998</v>
       </c>
     </row>
-    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>2026</v>
       </c>
@@ -2499,7 +2524,7 @@
         <v>138750.47</v>
       </c>
     </row>
-    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>2026</v>
       </c>
@@ -2516,7 +2541,7 @@
         <v>44182.25</v>
       </c>
     </row>
-    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>2026</v>
       </c>
@@ -2533,7 +2558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>2026</v>
       </c>
@@ -2550,7 +2575,7 @@
         <v>461.7826</v>
       </c>
     </row>
-    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>2026</v>
       </c>
@@ -2567,7 +2592,7 @@
         <v>2688.0174000000006</v>
       </c>
     </row>
-    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>2026</v>
       </c>
@@ -2584,7 +2609,7 @@
         <v>12739.311400000001</v>
       </c>
     </row>
-    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>2026</v>
       </c>
@@ -2601,7 +2626,7 @@
         <v>23679.965400000001</v>
       </c>
     </row>
-    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>2026</v>
       </c>
@@ -2618,7 +2643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>2026</v>
       </c>
@@ -2635,7 +2660,7 @@
         <v>77220.153899998884</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>2026</v>
       </c>
@@ -2652,7 +2677,7 @@
         <v>86121.755500000174</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>2026</v>
       </c>
@@ -2669,7 +2694,7 @@
         <v>173324.40840000182</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>2026</v>
       </c>
@@ -2686,7 +2711,7 @@
         <v>209302.24539999786</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>2026</v>
       </c>
@@ -2705,7 +2730,7 @@
       <c r="H126" s="1"/>
       <c r="I126" s="2"/>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>2026</v>
       </c>
@@ -2724,7 +2749,7 @@
       <c r="H127" s="1"/>
       <c r="I127" s="2"/>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>2026</v>
       </c>
@@ -2744,7 +2769,7 @@
       <c r="H128" s="1"/>
       <c r="I128" s="2"/>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>2026</v>
       </c>
@@ -2764,7 +2789,7 @@
       <c r="H129" s="1"/>
       <c r="I129" s="2"/>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>2026</v>
       </c>
@@ -2784,7 +2809,7 @@
       <c r="H130" s="1"/>
       <c r="I130" s="2"/>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>2026</v>
       </c>
@@ -2804,7 +2829,7 @@
       <c r="H131" s="1"/>
       <c r="I131" s="2"/>
     </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>2026</v>
       </c>
@@ -2824,7 +2849,7 @@
       <c r="H132" s="1"/>
       <c r="I132" s="2"/>
     </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>2026</v>
       </c>
@@ -2841,7 +2866,7 @@
         <v>181913.22</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>2026</v>
       </c>
@@ -2859,7 +2884,7 @@
         <v>12874.3482</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>2026</v>
       </c>
@@ -2877,7 +2902,7 @@
         <v>13987.576800000001</v>
       </c>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>2026</v>
       </c>
@@ -2894,7 +2919,7 @@
         <v>30450.855</v>
       </c>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>2026</v>
       </c>
@@ -2912,7 +2937,7 @@
         <v>33929.697800000002</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>2026</v>
       </c>
@@ -2930,7 +2955,7 @@
         <v>168855.25</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>2026</v>
       </c>
@@ -2947,7 +2972,7 @@
         <v>46098.47</v>
       </c>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>2026</v>
       </c>
@@ -2964,7 +2989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>2026</v>
       </c>
@@ -2981,7 +3006,7 @@
         <v>567.72</v>
       </c>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>2026</v>
       </c>
@@ -2998,7 +3023,7 @@
         <v>5096.16</v>
       </c>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>2026</v>
       </c>
@@ -3015,7 +3040,7 @@
         <v>1616.03</v>
       </c>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>2026</v>
       </c>
@@ -3032,7 +3057,7 @@
         <v>25567.72</v>
       </c>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>2026</v>
       </c>
@@ -3049,7 +3074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>2026</v>
       </c>
@@ -3066,7 +3091,7 @@
         <v>89361.818099997603</v>
       </c>
     </row>
-    <row r="147" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>2026</v>
       </c>
@@ -3083,7 +3108,7 @@
         <v>107441.32280000077</v>
       </c>
     </row>
-    <row r="148" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>2026</v>
       </c>
@@ -3102,7 +3127,7 @@
       <c r="G148" s="1"/>
       <c r="H148" s="2"/>
     </row>
-    <row r="149" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>2026</v>
       </c>
@@ -3121,7 +3146,7 @@
       <c r="G149" s="1"/>
       <c r="H149" s="2"/>
     </row>
-    <row r="150" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>2026</v>
       </c>
@@ -3140,7 +3165,7 @@
       <c r="G150" s="1"/>
       <c r="H150" s="2"/>
     </row>
-    <row r="151" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>2026</v>
       </c>
@@ -3159,7 +3184,7 @@
       <c r="G151" s="1"/>
       <c r="H151" s="2"/>
     </row>
-    <row r="152" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>2026</v>
       </c>
@@ -3179,7 +3204,7 @@
       <c r="G152" s="1"/>
       <c r="H152" s="2"/>
     </row>
-    <row r="153" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>2026</v>
       </c>
@@ -3199,7 +3224,7 @@
       <c r="G153" s="1"/>
       <c r="H153" s="2"/>
     </row>
-    <row r="154" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>2026</v>
       </c>
@@ -3217,7 +3242,7 @@
         <v>119855.82850000999</v>
       </c>
     </row>
-    <row r="155" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>2026</v>
       </c>
@@ -3235,7 +3260,7 @@
         <v>273290.69730000698</v>
       </c>
     </row>
-    <row r="156" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>2026</v>
       </c>
@@ -3253,7 +3278,7 @@
         <v>559041.84450000012</v>
       </c>
     </row>
-    <row r="157" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>2026</v>
       </c>
@@ -3270,7 +3295,7 @@
         <v>212372.49</v>
       </c>
     </row>
-    <row r="158" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>2026</v>
       </c>
@@ -3287,7 +3312,7 @@
         <v>12777.495299999999</v>
       </c>
     </row>
-    <row r="159" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>2026</v>
       </c>
@@ -3304,7 +3329,7 @@
         <v>13841.474399999999</v>
       </c>
     </row>
-    <row r="160" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>2026</v>
       </c>
@@ -3321,7 +3346,7 @@
         <v>31073.3325</v>
       </c>
     </row>
-    <row r="161" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>2026</v>
       </c>
@@ -3338,7 +3363,7 @@
         <v>33015.147799999999</v>
       </c>
     </row>
-    <row r="162" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>2026</v>
       </c>
@@ -3355,7 +3380,7 @@
         <v>131765.28</v>
       </c>
     </row>
-    <row r="163" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>2026</v>
       </c>
@@ -3372,7 +3397,7 @@
         <v>52245.279999999999</v>
       </c>
     </row>
-    <row r="164" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>2026</v>
       </c>
@@ -3390,7 +3415,7 @@
       </c>
       <c r="F164" s="1"/>
     </row>
-    <row r="165" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>2026</v>
       </c>
@@ -3408,7 +3433,7 @@
       </c>
       <c r="F165" s="1"/>
     </row>
-    <row r="166" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>2026</v>
       </c>
@@ -3426,7 +3451,7 @@
       </c>
       <c r="F166" s="1"/>
     </row>
-    <row r="167" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>2026</v>
       </c>
@@ -3444,7 +3469,7 @@
       </c>
       <c r="F167" s="1"/>
     </row>
-    <row r="168" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>2026</v>
       </c>
@@ -3461,7 +3486,7 @@
         <v>27911.695899999992</v>
       </c>
     </row>
-    <row r="169" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>2026</v>
       </c>
@@ -3478,7 +3503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>2026</v>
       </c>
@@ -3497,7 +3522,7 @@
       <c r="G170" s="2"/>
       <c r="I170" s="5"/>
     </row>
-    <row r="171" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>2026</v>
       </c>
@@ -3515,7 +3540,7 @@
       </c>
       <c r="I171" s="5"/>
     </row>
-    <row r="172" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>2026</v>
       </c>
@@ -3533,7 +3558,7 @@
       </c>
       <c r="I172" s="5"/>
     </row>
-    <row r="173" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>2026</v>
       </c>
@@ -3551,7 +3576,7 @@
       </c>
       <c r="I173" s="5"/>
     </row>
-    <row r="174" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>2026</v>
       </c>
@@ -3569,7 +3594,7 @@
       </c>
       <c r="I174" s="5"/>
     </row>
-    <row r="175" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>2026</v>
       </c>
@@ -3587,7 +3612,7 @@
       </c>
       <c r="I175" s="5"/>
     </row>
-    <row r="176" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>2026</v>
       </c>
@@ -3604,7 +3629,7 @@
         <v>84178.304800000013</v>
       </c>
     </row>
-    <row r="177" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>2026</v>
       </c>
@@ -3621,7 +3646,7 @@
         <v>50958.239000000001</v>
       </c>
     </row>
-    <row r="178" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>2026</v>
       </c>
@@ -3638,7 +3663,7 @@
         <v>127581.61459999997</v>
       </c>
     </row>
-    <row r="179" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>2026</v>
       </c>
@@ -3656,7 +3681,7 @@
       </c>
       <c r="F179" s="2"/>
     </row>
-    <row r="180" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>2026</v>
       </c>
@@ -3673,7 +3698,7 @@
         <v>593254.59900000005</v>
       </c>
     </row>
-    <row r="181" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>2026</v>
       </c>
@@ -3690,7 +3715,7 @@
         <v>202194.79</v>
       </c>
     </row>
-    <row r="182" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>2026</v>
       </c>
@@ -3707,7 +3732,7 @@
         <v>12130.191999999999</v>
       </c>
     </row>
-    <row r="183" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>2026</v>
       </c>
@@ -3724,7 +3749,7 @@
         <v>13187.980199999998</v>
       </c>
     </row>
-    <row r="184" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>2026</v>
       </c>
@@ -3741,7 +3766,7 @@
         <v>28505.212499999998</v>
       </c>
     </row>
-    <row r="185" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>2026</v>
       </c>
@@ -3758,7 +3783,7 @@
         <v>32112.155299999999</v>
       </c>
     </row>
-    <row r="186" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>2026</v>
       </c>
@@ -3775,7 +3800,7 @@
         <v>121544.80000000002</v>
       </c>
     </row>
-    <row r="187" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>2026</v>
       </c>
@@ -3792,7 +3817,7 @@
         <v>42219.37</v>
       </c>
     </row>
-    <row r="188" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>2026</v>
       </c>
@@ -3809,7 +3834,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>2026</v>
       </c>
@@ -3826,7 +3851,7 @@
         <v>543.69760000000008</v>
       </c>
     </row>
-    <row r="190" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>2026</v>
       </c>
@@ -3843,7 +3868,7 @@
         <v>2551.955899999999</v>
       </c>
     </row>
-    <row r="191" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>2026</v>
       </c>
@@ -3860,7 +3885,7 @@
         <v>1164.2699</v>
       </c>
     </row>
-    <row r="192" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>2026</v>
       </c>
@@ -3877,7 +3902,7 @@
         <v>21328.843700000001</v>
       </c>
     </row>
-    <row r="193" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>2026</v>
       </c>
@@ -3895,7 +3920,7 @@
       </c>
       <c r="G193" s="1"/>
     </row>
-    <row r="194" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>2026</v>
       </c>
@@ -3913,7 +3938,7 @@
       </c>
       <c r="G194" s="1"/>
     </row>
-    <row r="195" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>2026</v>
       </c>
@@ -3931,7 +3956,7 @@
       </c>
       <c r="G195" s="1"/>
     </row>
-    <row r="196" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>2026</v>
       </c>
@@ -3949,7 +3974,7 @@
       </c>
       <c r="G196" s="1"/>
     </row>
-    <row r="197" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>2026</v>
       </c>
@@ -3967,7 +3992,7 @@
       </c>
       <c r="G197" s="1"/>
     </row>
-    <row r="198" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198">
         <v>2026</v>
       </c>
@@ -3985,7 +4010,7 @@
       </c>
       <c r="G198" s="1"/>
     </row>
-    <row r="199" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199">
         <v>2026</v>
       </c>
@@ -4003,7 +4028,7 @@
       </c>
       <c r="G199" s="1"/>
     </row>
-    <row r="200" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200">
         <v>2026</v>
       </c>
@@ -4021,7 +4046,7 @@
       </c>
       <c r="G200" s="1"/>
     </row>
-    <row r="201" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A201">
         <v>2026</v>
       </c>
@@ -4038,7 +4063,7 @@
         <v>320.46504567906788</v>
       </c>
     </row>
-    <row r="202" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A202">
         <v>2026</v>
       </c>
@@ -4055,7 +4080,7 @@
         <v>781.82266878491987</v>
       </c>
     </row>
-    <row r="203" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A203">
         <v>2026</v>
       </c>
@@ -4072,7 +4097,7 @@
         <v>1562.6147636858752</v>
       </c>
     </row>
-    <row r="204" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204">
         <v>2026</v>
       </c>
@@ -4089,7 +4114,7 @@
         <v>3711.1972636560722</v>
       </c>
     </row>
-    <row r="205" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A205">
         <v>2026</v>
       </c>
@@ -4106,7 +4131,7 @@
         <v>1218.9366680465741</v>
       </c>
     </row>
-    <row r="206" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A206">
         <v>2026</v>
       </c>
@@ -4123,7 +4148,7 @@
         <v>678.32137263825587</v>
       </c>
     </row>
-    <row r="207" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207">
         <v>2026</v>
       </c>
@@ -4140,7 +4165,7 @@
         <v>502.93018387411206</v>
       </c>
     </row>
-    <row r="208" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208">
         <v>2026</v>
       </c>
@@ -4157,7 +4182,7 @@
         <v>1226.9738115611026</v>
       </c>
     </row>
-    <row r="209" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A209">
         <v>2026</v>
       </c>
@@ -4174,7 +4199,7 @@
         <v>2452.3302650984624</v>
       </c>
     </row>
-    <row r="210" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A210">
         <v>2026</v>
       </c>
@@ -4191,7 +4216,7 @@
         <v>5824.2642914411435</v>
       </c>
     </row>
-    <row r="211" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A211">
         <v>2026</v>
       </c>
@@ -4208,7 +4233,7 @@
         <v>1912.9700753869256</v>
       </c>
     </row>
-    <row r="212" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A212">
         <v>2026</v>
       </c>
@@ -4225,7 +4250,7 @@
         <v>609.57059480822136</v>
       </c>
     </row>
-    <row r="213" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A213">
         <v>2026</v>
       </c>
@@ -4242,7 +4267,7 @@
         <v>451.95605460399236</v>
       </c>
     </row>
-    <row r="214" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A214">
         <v>2026</v>
       </c>
@@ -4259,7 +4284,7 @@
         <v>1102.6147579847468</v>
       </c>
     </row>
-    <row r="215" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A215">
         <v>2026</v>
       </c>
@@ -4276,7 +4301,7 @@
         <v>2203.7760841120894</v>
       </c>
     </row>
-    <row r="216" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216">
         <v>2026</v>
       </c>
@@ -4293,7 +4318,7 @@
         <v>5233.950147620385</v>
       </c>
     </row>
-    <row r="217" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A217">
         <v>2026</v>
       </c>
@@ -4310,7 +4335,7 @@
         <v>1719.0823608705666</v>
       </c>
     </row>
-    <row r="218" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A218">
         <v>2026</v>
       </c>
@@ -4327,7 +4352,7 @@
         <v>744.32500541888055</v>
       </c>
     </row>
-    <row r="219" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A219">
         <v>2026</v>
       </c>
@@ -4344,7 +4369,7 @@
         <v>551.86748779778145</v>
       </c>
     </row>
-    <row r="220" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A220">
         <v>2026</v>
       </c>
@@ -4361,7 +4386,7 @@
         <v>1346.3637234176927</v>
       </c>
     </row>
-    <row r="221" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221">
         <v>2026</v>
       </c>
@@ -4378,7 +4403,7 @@
         <v>2690.9527128105606</v>
       </c>
     </row>
-    <row r="222" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A222">
         <v>2026</v>
       </c>
@@ -4395,7 +4420,7 @@
         <v>6390.9906500909046</v>
       </c>
     </row>
-    <row r="223" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A223">
         <v>2026</v>
       </c>
@@ -4412,7 +4437,7 @@
         <v>2099.1104204641815</v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A224">
         <v>2026</v>
       </c>
@@ -4429,7 +4454,7 @@
         <v>528.99233987992443</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A225">
         <v>2026</v>
       </c>
@@ -4446,7 +4471,7 @@
         <v>392.21263768978685</v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A226">
         <v>2026</v>
       </c>
@@ -4463,7 +4488,7 @@
         <v>956.86170852121484</v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A227">
         <v>2026</v>
       </c>
@@ -4480,7 +4505,7 @@
         <v>1912.4621122392568</v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A228">
         <v>2026</v>
       </c>
@@ -4497,7 +4522,7 @@
         <v>4542.0818507094455</v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A229">
         <v>2026</v>
       </c>
@@ -4514,7 +4539,7 @@
         <v>1491.8393509603734</v>
       </c>
     </row>
-    <row r="230" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A230">
         <v>2026</v>
       </c>
@@ -4531,7 +4556,7 @@
         <v>774.4423733517865</v>
       </c>
     </row>
-    <row r="231" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A231">
         <v>2026</v>
       </c>
@@ -4548,7 +4573,7 @@
         <v>574.19751306793967</v>
       </c>
     </row>
-    <row r="232" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A232">
         <v>2026</v>
       </c>
@@ -4565,7 +4590,7 @@
         <v>1400.8411779361904</v>
       </c>
     </row>
-    <row r="233" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A233">
         <v>2026</v>
       </c>
@@ -4582,7 +4607,7 @@
         <v>2799.8358113921513</v>
       </c>
     </row>
-    <row r="234" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A234">
         <v>2026</v>
       </c>
@@ -4599,7 +4624,7 @@
         <v>6649.587117310527</v>
       </c>
     </row>
-    <row r="235" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A235">
         <v>2026</v>
       </c>
@@ -4616,7 +4641,7 @@
         <v>2184.0460069414066</v>
       </c>
     </row>
-    <row r="236" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A236">
         <v>2026</v>
       </c>
@@ -4633,7 +4658,7 @@
         <v>771.25047294941464</v>
       </c>
     </row>
-    <row r="237" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237">
         <v>2026</v>
       </c>
@@ -4650,7 +4675,7 @@
         <v>571.83093120714841</v>
       </c>
     </row>
-    <row r="238" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238">
         <v>2026</v>
       </c>
@@ -4667,7 +4692,7 @@
         <v>1395.0675456126366</v>
       </c>
     </row>
-    <row r="239" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A239">
         <v>2026</v>
       </c>
@@ -4684,7 +4709,7 @@
         <v>2788.2961573643383</v>
       </c>
     </row>
-    <row r="240" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A240">
         <v>2026</v>
       </c>
@@ -4701,7 +4726,7 @@
         <v>6622.1805335210984</v>
       </c>
     </row>
-    <row r="241" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A241">
         <v>2026</v>
       </c>
@@ -4716,13 +4741,527 @@
       </c>
       <c r="E241" s="3">
         <v>2175.0443593453647</v>
+      </c>
+    </row>
+    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A243">
+        <v>2026</v>
+      </c>
+      <c r="B243" t="s">
+        <v>25</v>
+      </c>
+      <c r="C243" t="s">
+        <v>1</v>
+      </c>
+      <c r="D243" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E243">
+        <v>95728.084700000007</v>
+      </c>
+    </row>
+    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A244">
+        <v>2026</v>
+      </c>
+      <c r="B244" t="s">
+        <v>25</v>
+      </c>
+      <c r="C244" t="s">
+        <v>3</v>
+      </c>
+      <c r="D244" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E244" s="2">
+        <v>73499.102599999998</v>
+      </c>
+    </row>
+    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A245">
+        <v>2026</v>
+      </c>
+      <c r="B245" t="s">
+        <v>25</v>
+      </c>
+      <c r="C245" t="s">
+        <v>4</v>
+      </c>
+      <c r="D245" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E245" s="2">
+        <v>161766.7072</v>
+      </c>
+    </row>
+    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A246">
+        <v>2026</v>
+      </c>
+      <c r="B246" t="s">
+        <v>25</v>
+      </c>
+      <c r="C246" t="s">
+        <v>5</v>
+      </c>
+      <c r="D246" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E246" s="2">
+        <v>342906.08250000002</v>
+      </c>
+    </row>
+    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A247">
+        <v>2026</v>
+      </c>
+      <c r="B247" t="s">
+        <v>25</v>
+      </c>
+      <c r="C247" t="s">
+        <v>7</v>
+      </c>
+      <c r="D247" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E247" s="3">
+        <v>802815.92779994395</v>
+      </c>
+    </row>
+    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A248">
+        <v>2026</v>
+      </c>
+      <c r="B248" t="s">
+        <v>25</v>
+      </c>
+      <c r="C248" t="s">
+        <v>8</v>
+      </c>
+      <c r="D248" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E248" s="3">
+        <v>265105.07</v>
+      </c>
+    </row>
+    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A249">
+        <v>2026</v>
+      </c>
+      <c r="B249" t="s">
+        <v>25</v>
+      </c>
+      <c r="C249" t="s">
+        <v>1</v>
+      </c>
+      <c r="D249" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E249" s="2">
+        <v>90250.578400000013</v>
+      </c>
+    </row>
+    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A250">
+        <v>2026</v>
+      </c>
+      <c r="B250" t="s">
+        <v>25</v>
+      </c>
+      <c r="C250" t="s">
+        <v>3</v>
+      </c>
+      <c r="D250" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E250" s="2">
+        <v>62663.806999999993</v>
+      </c>
+    </row>
+    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A251">
+        <v>2026</v>
+      </c>
+      <c r="B251" t="s">
+        <v>25</v>
+      </c>
+      <c r="C251" t="s">
+        <v>4</v>
+      </c>
+      <c r="D251" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E251" s="2">
+        <v>149502.7254</v>
+      </c>
+    </row>
+    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A252">
+        <v>2026</v>
+      </c>
+      <c r="B252" t="s">
+        <v>25</v>
+      </c>
+      <c r="C252" t="s">
+        <v>5</v>
+      </c>
+      <c r="D252" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E252" s="2">
+        <v>300126.09499999997</v>
+      </c>
+    </row>
+    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A253">
+        <v>2026</v>
+      </c>
+      <c r="B253" t="s">
+        <v>25</v>
+      </c>
+      <c r="C253" t="s">
+        <v>7</v>
+      </c>
+      <c r="D253" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E253" s="2">
+        <v>609632.1459</v>
+      </c>
+    </row>
+    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A254">
+        <v>2026</v>
+      </c>
+      <c r="B254" t="s">
+        <v>25</v>
+      </c>
+      <c r="C254" t="s">
+        <v>8</v>
+      </c>
+      <c r="D254" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E254" s="3">
+        <v>213001.78</v>
+      </c>
+    </row>
+    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A255">
+        <v>2026</v>
+      </c>
+      <c r="B255" t="s">
+        <v>25</v>
+      </c>
+      <c r="C255" t="s">
+        <v>1</v>
+      </c>
+      <c r="D255" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E255">
+        <v>13582.3495</v>
+      </c>
+    </row>
+    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A256">
+        <v>2026</v>
+      </c>
+      <c r="B256" t="s">
+        <v>25</v>
+      </c>
+      <c r="C256" t="s">
+        <v>3</v>
+      </c>
+      <c r="D256" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E256" s="3">
+        <v>8889.4673999999995</v>
+      </c>
+    </row>
+    <row r="257" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A257">
+        <v>2026</v>
+      </c>
+      <c r="B257" t="s">
+        <v>25</v>
+      </c>
+      <c r="C257" t="s">
+        <v>4</v>
+      </c>
+      <c r="D257" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E257" s="3">
+        <v>32415.927599999999</v>
+      </c>
+    </row>
+    <row r="258" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A258">
+        <v>2026</v>
+      </c>
+      <c r="B258" t="s">
+        <v>25</v>
+      </c>
+      <c r="C258" t="s">
+        <v>5</v>
+      </c>
+      <c r="D258" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E258" s="3">
+        <v>33088.573100000001</v>
+      </c>
+      <c r="G258">
+        <f>49385.93*0.15</f>
+        <v>7407.8894999999993</v>
+      </c>
+    </row>
+    <row r="259" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A259">
+        <v>2026</v>
+      </c>
+      <c r="B259" t="s">
+        <v>25</v>
+      </c>
+      <c r="C259" t="s">
+        <v>7</v>
+      </c>
+      <c r="D259" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E259" s="3">
+        <v>127067.23</v>
+      </c>
+    </row>
+    <row r="260" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A260">
+        <v>2026</v>
+      </c>
+      <c r="B260" t="s">
+        <v>25</v>
+      </c>
+      <c r="C260" t="s">
+        <v>8</v>
+      </c>
+      <c r="D260" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E260" s="3">
+        <v>43717.19</v>
+      </c>
+    </row>
+    <row r="261" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A261">
+        <v>2026</v>
+      </c>
+      <c r="B261" t="s">
+        <v>25</v>
+      </c>
+      <c r="C261" t="s">
+        <v>1</v>
+      </c>
+      <c r="D261" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E261" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="262" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A262">
+        <v>2026</v>
+      </c>
+      <c r="B262" t="s">
+        <v>25</v>
+      </c>
+      <c r="C262" t="s">
+        <v>3</v>
+      </c>
+      <c r="D262" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E262" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="263" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A263">
+        <v>2026</v>
+      </c>
+      <c r="B263" t="s">
+        <v>25</v>
+      </c>
+      <c r="C263" t="s">
+        <v>4</v>
+      </c>
+      <c r="D263" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E263" s="3">
+        <v>4630.57</v>
+      </c>
+    </row>
+    <row r="264" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A264">
+        <v>2026</v>
+      </c>
+      <c r="B264" t="s">
+        <v>25</v>
+      </c>
+      <c r="C264" t="s">
+        <v>5</v>
+      </c>
+      <c r="D264" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E264" s="3">
+        <v>820.35</v>
+      </c>
+    </row>
+    <row r="265" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A265">
+        <v>2026</v>
+      </c>
+      <c r="B265" t="s">
+        <v>25</v>
+      </c>
+      <c r="C265" t="s">
+        <v>7</v>
+      </c>
+      <c r="D265" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E265" s="3">
+        <v>25743.1</v>
+      </c>
+    </row>
+    <row r="266" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A266">
+        <v>2026</v>
+      </c>
+      <c r="B266" t="s">
+        <v>25</v>
+      </c>
+      <c r="C266" t="s">
+        <v>8</v>
+      </c>
+      <c r="D266" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E266" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="267" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A267">
+        <v>2026</v>
+      </c>
+      <c r="B267" t="s">
+        <v>25</v>
+      </c>
+      <c r="C267" t="s">
+        <v>1</v>
+      </c>
+      <c r="D267" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E267" s="3">
+        <v>779.79250000000002</v>
+      </c>
+    </row>
+    <row r="268" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A268">
+        <v>2026</v>
+      </c>
+      <c r="B268" t="s">
+        <v>25</v>
+      </c>
+      <c r="C268" t="s">
+        <v>3</v>
+      </c>
+      <c r="D268" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E268" s="3">
+        <v>484.01099999999997</v>
+      </c>
+    </row>
+    <row r="269" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A269">
+        <v>2026</v>
+      </c>
+      <c r="B269" t="s">
+        <v>25</v>
+      </c>
+      <c r="C269" t="s">
+        <v>4</v>
+      </c>
+      <c r="D269" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E269">
+        <v>2312.4969999999998</v>
+      </c>
+    </row>
+    <row r="270" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A270">
+        <v>2026</v>
+      </c>
+      <c r="B270" t="s">
+        <v>25</v>
+      </c>
+      <c r="C270" t="s">
+        <v>5</v>
+      </c>
+      <c r="D270" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E270" s="3">
+        <v>1801.5964999999999</v>
+      </c>
+    </row>
+    <row r="271" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A271">
+        <v>2026</v>
+      </c>
+      <c r="B271" t="s">
+        <v>25</v>
+      </c>
+      <c r="C271" t="s">
+        <v>7</v>
+      </c>
+      <c r="D271" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E271" s="3">
+        <v>5377.09</v>
+      </c>
+    </row>
+    <row r="272" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A272">
+        <v>2026</v>
+      </c>
+      <c r="B272" t="s">
+        <v>25</v>
+      </c>
+      <c r="C272" t="s">
+        <v>8</v>
+      </c>
+      <c r="D272" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E272" s="3">
+        <v>2688.95</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E241" xr:uid="{1A73EA3A-E1FE-485B-B71A-B3ECBB4FF369}">
     <filterColumn colId="1">
       <filters>
-        <filter val="JUNIO"/>
+        <filter val="AGOSTO"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -4733,10 +5272,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D93FD4D-DA47-4482-8314-53DA1C6D364D}">
-  <dimension ref="A1:E49"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E55"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -4753,7 +5292,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2026</v>
       </c>
@@ -4770,7 +5309,7 @@
         <v>1205.39966</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2026</v>
       </c>
@@ -4787,7 +5326,7 @@
         <v>1049.8642199999999</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -4804,7 +5343,7 @@
         <v>2916.2894999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2026</v>
       </c>
@@ -4821,7 +5360,7 @@
         <v>2605.2186200000001</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2026</v>
       </c>
@@ -4838,7 +5377,7 @@
         <v>7776.7719999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2026</v>
       </c>
@@ -4855,7 +5394,7 @@
         <v>3888.386</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2026</v>
       </c>
@@ -4872,7 +5411,7 @@
         <v>944.99098000000004</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2026</v>
       </c>
@@ -4889,7 +5428,7 @@
         <v>823.05665999999997</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2026</v>
       </c>
@@ -4906,7 +5445,7 @@
         <v>2286.2685000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2026</v>
       </c>
@@ -4923,7 +5462,7 @@
         <v>2042.3998600000002</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2026</v>
       </c>
@@ -4940,7 +5479,7 @@
         <v>6096.7160000000003</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2026</v>
       </c>
@@ -4957,7 +5496,7 @@
         <v>3048.3580000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2026</v>
       </c>
@@ -4974,7 +5513,7 @@
         <v>944.99098000000004</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2026</v>
       </c>
@@ -4991,7 +5530,7 @@
         <v>823.05665999999997</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2026</v>
       </c>
@@ -5008,7 +5547,7 @@
         <v>2286.2685000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2026</v>
       </c>
@@ -5025,7 +5564,7 @@
         <v>2042.3998600000002</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2026</v>
       </c>
@@ -5042,7 +5581,7 @@
         <v>6096.7160000000003</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2026</v>
       </c>
@@ -5059,7 +5598,7 @@
         <v>3048.3580000000002</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2026</v>
       </c>
@@ -5076,7 +5615,7 @@
         <v>944.99098000000004</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2026</v>
       </c>
@@ -5093,7 +5632,7 @@
         <v>823.05665999999997</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2026</v>
       </c>
@@ -5110,7 +5649,7 @@
         <v>2286.2685000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2026</v>
       </c>
@@ -5127,7 +5666,7 @@
         <v>2042.3998600000002</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2026</v>
       </c>
@@ -5144,7 +5683,7 @@
         <v>6096.7160000000003</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2026</v>
       </c>
@@ -5161,7 +5700,7 @@
         <v>3048.3580000000002</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2026</v>
       </c>
@@ -5178,7 +5717,7 @@
         <v>2544.8643999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2026</v>
       </c>
@@ -5195,7 +5734,7 @@
         <v>2216.4947999999999</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2026</v>
       </c>
@@ -5212,7 +5751,7 @@
         <v>6156.93</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>2026</v>
       </c>
@@ -5229,7 +5768,7 @@
         <v>5500.1908000000003</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2026</v>
       </c>
@@ -5246,7 +5785,7 @@
         <v>16418.48</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2026</v>
       </c>
@@ -5263,7 +5802,7 @@
         <v>8209.24</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2026</v>
       </c>
@@ -5280,7 +5819,7 @@
         <v>2544.8643999999999</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2026</v>
       </c>
@@ -5297,7 +5836,7 @@
         <v>2216.4947999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2026</v>
       </c>
@@ -5314,7 +5853,7 @@
         <v>6156.93</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2026</v>
       </c>
@@ -5331,7 +5870,7 @@
         <v>5500.1908000000003</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>2026</v>
       </c>
@@ -5348,7 +5887,7 @@
         <v>16418.48</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>2026</v>
       </c>
@@ -5365,7 +5904,7 @@
         <v>8209.24</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>2026</v>
       </c>
@@ -5382,7 +5921,7 @@
         <v>2895.9889999999996</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2026</v>
       </c>
@@ -5399,7 +5938,7 @@
         <v>2522.3130000000001</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>2026</v>
       </c>
@@ -5416,7 +5955,7 @@
         <v>7006.4249999999993</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>2026</v>
       </c>
@@ -5433,7 +5972,7 @@
         <v>6259.0730000000003</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>2026</v>
       </c>
@@ -5450,7 +5989,7 @@
         <v>18683.8</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>2026</v>
       </c>
@@ -5467,7 +6006,7 @@
         <v>9341.9</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>2026</v>
       </c>
@@ -5484,7 +6023,7 @@
         <v>1693.2819999999999</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>2026</v>
       </c>
@@ -5501,7 +6040,7 @@
         <v>1474.7939999999999</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>2026</v>
       </c>
@@ -5518,7 +6057,7 @@
         <v>4096.6499999999996</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>2026</v>
       </c>
@@ -5535,7 +6074,7 @@
         <v>3659.674</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2026</v>
       </c>
@@ -5552,7 +6091,7 @@
         <v>10924.4</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>2026</v>
       </c>
@@ -5566,6 +6105,108 @@
         <v>9</v>
       </c>
       <c r="E49">
+        <v>5462.2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>2026</v>
+      </c>
+      <c r="B50" t="s">
+        <v>25</v>
+      </c>
+      <c r="C50" t="s">
+        <v>1</v>
+      </c>
+      <c r="D50" t="s">
+        <v>9</v>
+      </c>
+      <c r="E50">
+        <v>1693.2819999999999</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>2026</v>
+      </c>
+      <c r="B51" t="s">
+        <v>25</v>
+      </c>
+      <c r="C51" t="s">
+        <v>3</v>
+      </c>
+      <c r="D51" t="s">
+        <v>9</v>
+      </c>
+      <c r="E51">
+        <v>1474.7939999999999</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>2026</v>
+      </c>
+      <c r="B52" t="s">
+        <v>25</v>
+      </c>
+      <c r="C52" t="s">
+        <v>4</v>
+      </c>
+      <c r="D52" t="s">
+        <v>9</v>
+      </c>
+      <c r="E52">
+        <v>4096.6499999999996</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>2026</v>
+      </c>
+      <c r="B53" t="s">
+        <v>25</v>
+      </c>
+      <c r="C53" t="s">
+        <v>5</v>
+      </c>
+      <c r="D53" t="s">
+        <v>9</v>
+      </c>
+      <c r="E53">
+        <v>3659.674</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>2026</v>
+      </c>
+      <c r="B54" t="s">
+        <v>25</v>
+      </c>
+      <c r="C54" t="s">
+        <v>7</v>
+      </c>
+      <c r="D54" t="s">
+        <v>9</v>
+      </c>
+      <c r="E54">
+        <v>10924.4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>2026</v>
+      </c>
+      <c r="B55" t="s">
+        <v>25</v>
+      </c>
+      <c r="C55" t="s">
+        <v>8</v>
+      </c>
+      <c r="D55" t="s">
+        <v>9</v>
+      </c>
+      <c r="E55">
         <v>5462.2</v>
       </c>
     </row>

</xml_diff>